<commit_message>
Major Reorganization and Cleanup Before Review
</commit_message>
<xml_diff>
--- a/Predictions/2026-08-29.xlsx
+++ b/Predictions/2026-08-29.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdsak\OneDrive\Desktop\UFC ML\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gdsak\OneDrive\Desktop\UFC ML\Predictions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F703D959-A04D-42C8-8741-ACCD2515EF2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F54159B-F853-4B6A-BFCE-95F945361517}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -200,7 +200,7 @@
       <name val="Calibri"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -211,6 +211,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD3D3D3"/>
         <bgColor rgb="FFD3D3D3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -241,7 +253,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -250,6 +262,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -698,16 +719,16 @@
       <c r="E3" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="3">
+      <c r="G3" s="5">
         <v>0.61577953884116998</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H3" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="3">
+      <c r="I3" s="5">
         <v>0.51608891894125497</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -719,7 +740,7 @@
       <c r="L3" s="3">
         <v>0.40525586863934659</v>
       </c>
-      <c r="M3" s="3">
+      <c r="M3" s="6">
         <v>0.25980636381548322</v>
       </c>
       <c r="N3" s="3">
@@ -751,22 +772,22 @@
       <c r="E4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G4" s="3">
+      <c r="G4" s="5">
         <v>0.50890052278940801</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="3">
+      <c r="I4" s="5">
         <v>0.66575491914369433</v>
       </c>
-      <c r="J4" s="2" t="s">
+      <c r="J4" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="K4" s="3">
+      <c r="K4" s="5">
         <v>0.42226072817489763</v>
       </c>
       <c r="L4" s="3">
@@ -804,22 +825,22 @@
       <c r="E5" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G5" s="3">
+      <c r="G5" s="5">
         <v>0.50799963675013116</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="H5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="I5" s="3">
+      <c r="I5" s="5">
         <v>0.58447242498942853</v>
       </c>
-      <c r="J5" s="2" t="s">
+      <c r="J5" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="K5" s="3">
+      <c r="K5" s="5">
         <v>0.44054183801091717</v>
       </c>
       <c r="L5" s="3">
@@ -857,22 +878,22 @@
       <c r="E6" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="5">
         <v>0.78722243941813563</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I6" s="3">
+      <c r="I6" s="5">
         <v>0.82757980427337396</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J6" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="K6" s="3">
+      <c r="K6" s="5">
         <v>0.51184950048494327</v>
       </c>
       <c r="L6" s="3">
@@ -910,22 +931,22 @@
       <c r="E7" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="G7" s="3">
+      <c r="G7" s="5">
         <v>0.53657626368706901</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="I7" s="3">
+      <c r="I7" s="5">
         <v>0.55623439711543232</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="K7" s="3">
+      <c r="K7" s="5">
         <v>0.44853204370300231</v>
       </c>
       <c r="L7" s="3">
@@ -963,16 +984,16 @@
       <c r="E8" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="G8" s="3">
+      <c r="G8" s="5">
         <v>0.78513511473368336</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="I8" s="3">
+      <c r="I8" s="5">
         <v>0.7351091817147718</v>
       </c>
       <c r="J8" s="2" t="s">
@@ -984,7 +1005,7 @@
       <c r="L8" s="3">
         <v>0.44832163950442011</v>
       </c>
-      <c r="M8" s="3">
+      <c r="M8" s="6">
         <v>0.28891448446164342</v>
       </c>
       <c r="N8" s="3">

</xml_diff>